<commit_message>
Finalize Tier 1 operating review workbook, correct delivery record and remove temporary transport workflow
</commit_message>
<xml_diff>
--- a/enterprise/operations/publications/operating-review-v1.0.0.xlsx
+++ b/enterprise/operations/publications/operating-review-v1.0.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" r:id="R245f7d02dc914767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash obligations" sheetId="2" r:id="R8e19963945ec424d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control reviews" sheetId="3" r:id="R31bb912ce58b4ef8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer ARR" sheetId="4" r:id="R1939cf670f1b460a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial source" sheetId="5" r:id="R8cbf78d9ecf5447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast review" sheetId="6" r:id="R07dbbaca7d994ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" r:id="R18f9eef44362429f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash obligations" sheetId="2" r:id="R6c5a7243425b4d8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control reviews" sheetId="3" r:id="R248500f8f50a43a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer ARR" sheetId="4" r:id="R8a4e55dafd7b4523"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial source" sheetId="5" r:id="R7e63ab0049734ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast review" sheetId="6" r:id="R75a2e38ec6584104"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -147,7 +147,7 @@
         <x:color rgb="FFA32020"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4E4"/>
         </x:patternFill>
       </x:fill>
@@ -158,7 +158,7 @@
         <x:color rgb="FFA32020"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4E4"/>
         </x:patternFill>
       </x:fill>
@@ -168,7 +168,7 @@
         <x:color rgb="FF8A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D1"/>
         </x:patternFill>
       </x:fill>
@@ -179,7 +179,7 @@
         <x:color rgb="FFA32020"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4E4"/>
         </x:patternFill>
       </x:fill>
@@ -190,7 +190,7 @@
         <x:color rgb="FFA32020"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4E4"/>
         </x:patternFill>
       </x:fill>
@@ -488,19 +488,19 @@
       </x:c>
       <x:c r="E6" s="22" t="n">
         <x:f>SUMIFS('Financial source'!$D$6:$D$167,'Financial source'!$A$6:$A$167,$C6,'Financial source'!$B$6:$B$167,$D6,'Financial source'!$C$6:$C$167,$D$3)</x:f>
-        <x:v>10030080</x:v>
+        <x:v>9971200</x:v>
       </x:c>
       <x:c r="F6" s="22" t="n">
         <x:f>SUMIFS('Financial source'!$E$6:$E$167,'Financial source'!$A$6:$A$167,$C6,'Financial source'!$B$6:$B$167,$D6,'Financial source'!$C$6:$C$167,$D$3)</x:f>
-        <x:v>5256712.8128</x:v>
+        <x:v>5256508.0128</x:v>
       </x:c>
       <x:c r="G6" s="22" t="n">
         <x:f>SUMIFS('Financial source'!$F$6:$F$167,'Financial source'!$A$6:$A$167,$C6,'Financial source'!$B$6:$B$167,$D6,'Financial source'!$C$6:$C$167,$D$3)</x:f>
-        <x:v>4773367.1872</x:v>
+        <x:v>4714691.9872</x:v>
       </x:c>
       <x:c r="H6" s="22" t="n">
         <x:f>SUMIFS('Financial source'!$J$6:$J$167,'Financial source'!$A$6:$A$167,$C6,'Financial source'!$B$6:$B$167,$D6,'Financial source'!$C$6:$C$167,$D$3)</x:f>
-        <x:v>5447219.9872</x:v>
+        <x:v>5398579.9872</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
@@ -540,19 +540,19 @@
       </x:c>
       <x:c r="E8" s="13" t="n">
         <x:f>SUMIFS('Financial source'!$D$6:$D$167,'Financial source'!$A$6:$A$167,$C8,'Financial source'!$B$6:$B$167,$D8,'Financial source'!$C$6:$C$167,$D$3)</x:f>
-        <x:v>10982400</x:v>
+        <x:v>10810176</x:v>
       </x:c>
       <x:c r="F8" s="13" t="n">
         <x:f>SUMIFS('Financial source'!$E$6:$E$167,'Financial source'!$A$6:$A$167,$C8,'Financial source'!$B$6:$B$167,$D8,'Financial source'!$C$6:$C$167,$D$3)</x:f>
-        <x:v>5495001.3952</x:v>
+        <x:v>5494402.3552</x:v>
       </x:c>
       <x:c r="G8" s="13" t="n">
         <x:f>SUMIFS('Financial source'!$F$6:$F$167,'Financial source'!$A$6:$A$167,$C8,'Financial source'!$B$6:$B$167,$D8,'Financial source'!$C$6:$C$167,$D$3)</x:f>
-        <x:v>5487398.6048</x:v>
+        <x:v>5315773.6448</x:v>
       </x:c>
       <x:c r="H8" s="13" t="n">
         <x:f>SUMIFS('Financial source'!$J$6:$J$167,'Financial source'!$A$6:$A$167,$C8,'Financial source'!$B$6:$B$167,$D8,'Financial source'!$C$6:$C$167,$D$3)</x:f>
-        <x:v>6097001.6768</x:v>
+        <x:v>5954729.6768</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -1264,7 +1264,7 @@
     </x:row>
     <x:row r="4" ht="19" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Content: edd301ad6c9d319532dfd9ae79ecdbfd5456fa73aeec8e61da1ca6f9279317ac</x:v>
+        <x:v>Content: 5e302a4ba1b5c7c5678f4e3ee599b7f72029c4d58271dd47c6d3992541226bb2</x:v>
       </x:c>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1"/>
@@ -2714,7 +2714,7 @@
     </x:row>
     <x:row r="4" ht="19" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Content: edd301ad6c9d319532dfd9ae79ecdbfd5456fa73aeec8e61da1ca6f9279317ac</x:v>
+        <x:v>Content: 5e302a4ba1b5c7c5678f4e3ee599b7f72029c4d58271dd47c6d3992541226bb2</x:v>
       </x:c>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1"/>
@@ -6229,7 +6229,7 @@
     </x:row>
     <x:row r="4" ht="19" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Content: edd301ad6c9d319532dfd9ae79ecdbfd5456fa73aeec8e61da1ca6f9279317ac</x:v>
+        <x:v>Content: 5e302a4ba1b5c7c5678f4e3ee599b7f72029c4d58271dd47c6d3992541226bb2</x:v>
       </x:c>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1"/>
@@ -7425,7 +7425,7 @@
     </x:row>
     <x:row r="4" ht="19" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Content: edd301ad6c9d319532dfd9ae79ecdbfd5456fa73aeec8e61da1ca6f9279317ac</x:v>
+        <x:v>Content: 5e302a4ba1b5c7c5678f4e3ee599b7f72029c4d58271dd47c6d3992541226bb2</x:v>
       </x:c>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1"/>
@@ -7512,25 +7512,25 @@
         <x:v>2027</x:v>
       </x:c>
       <x:c r="D7" s="13" t="n">
-        <x:v>10030080</x:v>
+        <x:v>9971200</x:v>
       </x:c>
       <x:c r="E7" s="13" t="n">
-        <x:v>5256712.8128</x:v>
+        <x:v>5256508.0128</x:v>
       </x:c>
       <x:c r="F7" s="13" t="n">
-        <x:v>4773367.1872</x:v>
+        <x:v>4714691.9872</x:v>
       </x:c>
       <x:c r="G7" s="13" t="n">
-        <x:v>6644766.1872</x:v>
+        <x:v>6586090.9872</x:v>
       </x:c>
       <x:c r="H7" s="13" t="n">
         <x:v>1908464</x:v>
       </x:c>
       <x:c r="I7" s="13" t="n">
-        <x:v>4736302.1872</x:v>
+        <x:v>4677626.9872</x:v>
       </x:c>
       <x:c r="J7" s="13" t="n">
-        <x:v>5447219.9872</x:v>
+        <x:v>5398579.9872</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="19" customHeight="1">
@@ -7544,25 +7544,25 @@
         <x:v>2028</x:v>
       </x:c>
       <x:c r="D8" s="13" t="n">
-        <x:v>12874080</x:v>
+        <x:v>12776800</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
         <x:v>5453416.0128</x:v>
       </x:c>
       <x:c r="F8" s="13" t="n">
-        <x:v>7420663.9872</x:v>
+        <x:v>7323383.9872</x:v>
       </x:c>
       <x:c r="G8" s="13" t="n">
-        <x:v>14065430.1744</x:v>
+        <x:v>13909474.9744</x:v>
       </x:c>
       <x:c r="H8" s="13" t="n">
         <x:v>1908464</x:v>
       </x:c>
       <x:c r="I8" s="13" t="n">
-        <x:v>12156966.1744</x:v>
+        <x:v>12001010.9744</x:v>
       </x:c>
       <x:c r="J8" s="13" t="n">
-        <x:v>12867883.9744</x:v>
+        <x:v>12721963.9744</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="19" customHeight="1">
@@ -7576,25 +7576,25 @@
         <x:v>2029</x:v>
       </x:c>
       <x:c r="D9" s="13" t="n">
-        <x:v>12874080</x:v>
+        <x:v>12776800</x:v>
       </x:c>
       <x:c r="E9" s="13" t="n">
         <x:v>5609461.0128</x:v>
       </x:c>
       <x:c r="F9" s="13" t="n">
-        <x:v>7264618.9872</x:v>
+        <x:v>7167338.9872</x:v>
       </x:c>
       <x:c r="G9" s="13" t="n">
-        <x:v>21330049.1616</x:v>
+        <x:v>21076813.9616</x:v>
       </x:c>
       <x:c r="H9" s="13" t="n">
         <x:v>1908464</x:v>
       </x:c>
       <x:c r="I9" s="13" t="n">
-        <x:v>19421585.1616</x:v>
+        <x:v>19168349.9616</x:v>
       </x:c>
       <x:c r="J9" s="13" t="n">
-        <x:v>20132502.9616</x:v>
+        <x:v>19889302.9616</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="19" customHeight="1">
@@ -7608,25 +7608,25 @@
         <x:v>2030</x:v>
       </x:c>
       <x:c r="D10" s="13" t="n">
-        <x:v>12874080</x:v>
+        <x:v>12776800</x:v>
       </x:c>
       <x:c r="E10" s="13" t="n">
         <x:v>5770187.3436</x:v>
       </x:c>
       <x:c r="F10" s="13" t="n">
-        <x:v>7103892.6564</x:v>
+        <x:v>7006612.6564</x:v>
       </x:c>
       <x:c r="G10" s="13" t="n">
-        <x:v>28433941.818</x:v>
+        <x:v>28083426.618</x:v>
       </x:c>
       <x:c r="H10" s="13" t="n">
         <x:v>1908464</x:v>
       </x:c>
       <x:c r="I10" s="13" t="n">
-        <x:v>26525477.818</x:v>
+        <x:v>26174962.618</x:v>
       </x:c>
       <x:c r="J10" s="13" t="n">
-        <x:v>27236395.618</x:v>
+        <x:v>26895915.618</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="19" customHeight="1">
@@ -7640,25 +7640,25 @@
         <x:v>2031</x:v>
       </x:c>
       <x:c r="D11" s="13" t="n">
-        <x:v>12874080</x:v>
+        <x:v>12776800</x:v>
       </x:c>
       <x:c r="E11" s="13" t="n">
         <x:v>5935735.4784</x:v>
       </x:c>
       <x:c r="F11" s="13" t="n">
-        <x:v>6938344.5216</x:v>
+        <x:v>6841064.5216</x:v>
       </x:c>
       <x:c r="G11" s="13" t="n">
-        <x:v>35372286.3396</x:v>
+        <x:v>34924491.1396</x:v>
       </x:c>
       <x:c r="H11" s="13" t="n">
         <x:v>1908464</x:v>
       </x:c>
       <x:c r="I11" s="13" t="n">
-        <x:v>33463822.3396</x:v>
+        <x:v>33016027.1396</x:v>
       </x:c>
       <x:c r="J11" s="13" t="n">
-        <x:v>34174740.1396</x:v>
+        <x:v>33736980.1396</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="19" customHeight="1">
@@ -8129,16 +8129,16 @@
         <x:v>-39180334.2724</x:v>
       </x:c>
       <x:c r="G26" s="13" t="n">
-        <x:v>217913491.8643</x:v>
+        <x:v>217972371.8643</x:v>
       </x:c>
       <x:c r="H26" s="13" t="n">
         <x:v>31727485.7668</x:v>
       </x:c>
       <x:c r="I26" s="13" t="n">
-        <x:v>186186006.0975</x:v>
+        <x:v>186244886.0975</x:v>
       </x:c>
       <x:c r="J26" s="13" t="n">
-        <x:v>-56839659.2528</x:v>
+        <x:v>-56780779.2528</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="19" customHeight="1">
@@ -8161,16 +8161,16 @@
         <x:v>-40157363.2724</x:v>
       </x:c>
       <x:c r="G27" s="13" t="n">
-        <x:v>176556128.5919</x:v>
+        <x:v>176615008.5919</x:v>
       </x:c>
       <x:c r="H27" s="13" t="n">
         <x:v>30527485.7668</x:v>
       </x:c>
       <x:c r="I27" s="13" t="n">
-        <x:v>146028642.8251</x:v>
+        <x:v>146087522.8251</x:v>
       </x:c>
       <x:c r="J27" s="13" t="n">
-        <x:v>-97265848.2004</x:v>
+        <x:v>-97206968.2004</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="19" customHeight="1">
@@ -8193,16 +8193,16 @@
         <x:v>-41139520.7504</x:v>
       </x:c>
       <x:c r="G28" s="13" t="n">
-        <x:v>134216607.8415</x:v>
+        <x:v>134275487.8415</x:v>
       </x:c>
       <x:c r="H28" s="13" t="n">
         <x:v>29327485.7668</x:v>
       </x:c>
       <x:c r="I28" s="13" t="n">
-        <x:v>104889122.0747</x:v>
+        <x:v>104948002.0747</x:v>
       </x:c>
       <x:c r="J28" s="13" t="n">
-        <x:v>-138686925.426</x:v>
+        <x:v>-138628045.426</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="19" customHeight="1">
@@ -8225,16 +8225,16 @@
         <x:v>-42153482.7284</x:v>
       </x:c>
       <x:c r="G29" s="13" t="n">
-        <x:v>90863125.1131</x:v>
+        <x:v>90922005.1131</x:v>
       </x:c>
       <x:c r="H29" s="13" t="n">
         <x:v>28127485.7668</x:v>
       </x:c>
       <x:c r="I29" s="13" t="n">
-        <x:v>62735639.3463</x:v>
+        <x:v>62794519.3463</x:v>
       </x:c>
       <x:c r="J29" s="13" t="n">
-        <x:v>-181135077.3536</x:v>
+        <x:v>-181076197.3536</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="19" customHeight="1">
@@ -10968,25 +10968,25 @@
         <x:v>2027</x:v>
       </x:c>
       <x:c r="D115" s="13" t="n">
-        <x:v>10982400</x:v>
+        <x:v>10810176</x:v>
       </x:c>
       <x:c r="E115" s="13" t="n">
-        <x:v>5495001.3952</x:v>
+        <x:v>5494402.3552</x:v>
       </x:c>
       <x:c r="F115" s="13" t="n">
-        <x:v>5487398.6048</x:v>
+        <x:v>5315773.6448</x:v>
       </x:c>
       <x:c r="G115" s="13" t="n">
-        <x:v>7417980.8368</x:v>
+        <x:v>7246355.8768</x:v>
       </x:c>
       <x:c r="H115" s="13" t="n">
         <x:v>1967647.232</x:v>
       </x:c>
       <x:c r="I115" s="13" t="n">
-        <x:v>5450333.6048</x:v>
+        <x:v>5278708.6448</x:v>
       </x:c>
       <x:c r="J115" s="13" t="n">
-        <x:v>6097001.6768</x:v>
+        <x:v>5954729.6768</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="19" customHeight="1">
@@ -11000,25 +11000,25 @@
         <x:v>2028</x:v>
       </x:c>
       <x:c r="D116" s="13" t="n">
-        <x:v>14299584</x:v>
+        <x:v>14015040</x:v>
       </x:c>
       <x:c r="E116" s="13" t="n">
         <x:v>5702991.744</x:v>
       </x:c>
       <x:c r="F116" s="13" t="n">
-        <x:v>8596592.256</x:v>
+        <x:v>8312048.256</x:v>
       </x:c>
       <x:c r="G116" s="13" t="n">
-        <x:v>16014573.0928</x:v>
+        <x:v>15558404.1328</x:v>
       </x:c>
       <x:c r="H116" s="13" t="n">
         <x:v>1967647.232</x:v>
       </x:c>
       <x:c r="I116" s="13" t="n">
-        <x:v>14046925.8608</x:v>
+        <x:v>13590756.9008</x:v>
       </x:c>
       <x:c r="J116" s="13" t="n">
-        <x:v>14693593.9328</x:v>
+        <x:v>14266777.9328</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="19" customHeight="1">
@@ -11032,25 +11032,25 @@
         <x:v>2029</x:v>
       </x:c>
       <x:c r="D117" s="13" t="n">
-        <x:v>14299584</x:v>
+        <x:v>14015040</x:v>
       </x:c>
       <x:c r="E117" s="13" t="n">
         <x:v>5865278.544</x:v>
       </x:c>
       <x:c r="F117" s="13" t="n">
-        <x:v>8434305.456</x:v>
+        <x:v>8149761.456</x:v>
       </x:c>
       <x:c r="G117" s="13" t="n">
-        <x:v>24448878.5488</x:v>
+        <x:v>23708165.5888</x:v>
       </x:c>
       <x:c r="H117" s="13" t="n">
         <x:v>1967647.232</x:v>
       </x:c>
       <x:c r="I117" s="13" t="n">
-        <x:v>22481231.3168</x:v>
+        <x:v>21740518.3568</x:v>
       </x:c>
       <x:c r="J117" s="13" t="n">
-        <x:v>23127899.3888</x:v>
+        <x:v>22416539.3888</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="19" customHeight="1">
@@ -11064,25 +11064,25 @@
         <x:v>2030</x:v>
       </x:c>
       <x:c r="D118" s="13" t="n">
-        <x:v>14299584</x:v>
+        <x:v>14015040</x:v>
       </x:c>
       <x:c r="E118" s="13" t="n">
         <x:v>6032433.948</x:v>
       </x:c>
       <x:c r="F118" s="13" t="n">
-        <x:v>8267150.052</x:v>
+        <x:v>7982606.052</x:v>
       </x:c>
       <x:c r="G118" s="13" t="n">
-        <x:v>32716028.6008</x:v>
+        <x:v>31690771.6408</x:v>
       </x:c>
       <x:c r="H118" s="13" t="n">
         <x:v>1967647.232</x:v>
       </x:c>
       <x:c r="I118" s="13" t="n">
-        <x:v>30748381.3688</x:v>
+        <x:v>29723124.4088</x:v>
       </x:c>
       <x:c r="J118" s="13" t="n">
-        <x:v>31395049.4408</x:v>
+        <x:v>30399145.4408</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="19" customHeight="1">
@@ -11096,25 +11096,25 @@
         <x:v>2031</x:v>
       </x:c>
       <x:c r="D119" s="13" t="n">
-        <x:v>14299584</x:v>
+        <x:v>14015040</x:v>
       </x:c>
       <x:c r="E119" s="13" t="n">
         <x:v>6204604.0212</x:v>
       </x:c>
       <x:c r="F119" s="13" t="n">
-        <x:v>8094979.9788</x:v>
+        <x:v>7810435.9788</x:v>
       </x:c>
       <x:c r="G119" s="13" t="n">
-        <x:v>40811008.5796</x:v>
+        <x:v>39501207.6196</x:v>
       </x:c>
       <x:c r="H119" s="13" t="n">
         <x:v>1967647.232</x:v>
       </x:c>
       <x:c r="I119" s="13" t="n">
-        <x:v>38843361.3476</x:v>
+        <x:v>37533560.3876</x:v>
       </x:c>
       <x:c r="J119" s="13" t="n">
-        <x:v>39490029.4196</x:v>
+        <x:v>38209581.4196</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="19" customHeight="1">
@@ -12724,7 +12724,7 @@
     </x:row>
     <x:row r="4" ht="19" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Content: edd301ad6c9d319532dfd9ae79ecdbfd5456fa73aeec8e61da1ca6f9279317ac</x:v>
+        <x:v>Content: 5e302a4ba1b5c7c5678f4e3ee599b7f72029c4d58271dd47c6d3992541226bb2</x:v>
       </x:c>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1"/>
@@ -12793,16 +12793,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F6" s="13" t="n">
-        <x:v>4773367.1872</x:v>
+        <x:v>4714691.9872</x:v>
       </x:c>
       <x:c r="G6" s="13" t="n">
-        <x:v>5143509.7072</x:v>
+        <x:v>5083830.9872</x:v>
       </x:c>
       <x:c r="H6" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="13" t="n">
-        <x:v>370142.52</x:v>
+        <x:v>369139</x:v>
       </x:c>
       <x:c r="J6" s="13" t="n">
         <x:v>0</x:v>
@@ -12812,7 +12812,7 @@
       </x:c>
       <x:c r="L6" s="14" t="n">
         <x:f>G6-F6-SUM(H6:K6)</x:f>
-        <x:v>4.656612873077393e-10</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="19" customHeight="1">
@@ -12832,16 +12832,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F7" s="13" t="n">
-        <x:v>10030080</x:v>
+        <x:v>9971200</x:v>
       </x:c>
       <x:c r="G7" s="13" t="n">
-        <x:v>10410384</x:v>
+        <x:v>10350480</x:v>
       </x:c>
       <x:c r="H7" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I7" s="13" t="n">
-        <x:v>380304</x:v>
+        <x:v>379280</x:v>
       </x:c>
       <x:c r="J7" s="13" t="n">
         <x:v>0</x:v>
@@ -12871,10 +12871,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F8" s="13" t="n">
-        <x:v>5143509.7072</x:v>
+        <x:v>5083830.9872</x:v>
       </x:c>
       <x:c r="G8" s="13" t="n">
-        <x:v>5143509.7072</x:v>
+        <x:v>5083830.9872</x:v>
       </x:c>
       <x:c r="H8" s="13" t="n">
         <x:v>0</x:v>
@@ -12910,10 +12910,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F9" s="13" t="n">
-        <x:v>10410384</x:v>
+        <x:v>10350480</x:v>
       </x:c>
       <x:c r="G9" s="13" t="n">
-        <x:v>10410384</x:v>
+        <x:v>10350480</x:v>
       </x:c>
       <x:c r="H9" s="13" t="n">
         <x:v>0</x:v>
@@ -12949,16 +12949,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F10" s="13" t="n">
-        <x:v>7420663.9872</x:v>
+        <x:v>7323383.9872</x:v>
       </x:c>
       <x:c r="G10" s="13" t="n">
-        <x:v>8682880.3872</x:v>
+        <x:v>8575872.3872</x:v>
       </x:c>
       <x:c r="H10" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="13" t="n">
-        <x:v>1262216.4</x:v>
+        <x:v>1252488.4</x:v>
       </x:c>
       <x:c r="J10" s="13" t="n">
         <x:v>0</x:v>
@@ -12988,16 +12988,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F11" s="13" t="n">
-        <x:v>12874080</x:v>
+        <x:v>12776800</x:v>
       </x:c>
       <x:c r="G11" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="H11" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="13" t="n">
-        <x:v>1287408</x:v>
+        <x:v>1277680</x:v>
       </x:c>
       <x:c r="J11" s="13" t="n">
         <x:v>0</x:v>
@@ -13027,10 +13027,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F12" s="13" t="n">
-        <x:v>8682880.3872</x:v>
+        <x:v>8575872.3872</x:v>
       </x:c>
       <x:c r="G12" s="13" t="n">
-        <x:v>8682880.3872</x:v>
+        <x:v>8575872.3872</x:v>
       </x:c>
       <x:c r="H12" s="13" t="n">
         <x:v>0</x:v>
@@ -13066,10 +13066,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F13" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="G13" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="H13" s="13" t="n">
         <x:v>0</x:v>
@@ -13105,16 +13105,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F14" s="13" t="n">
-        <x:v>7264618.9872</x:v>
+        <x:v>7167338.9872</x:v>
       </x:c>
       <x:c r="G14" s="13" t="n">
-        <x:v>8526835.3872</x:v>
+        <x:v>8419827.3872</x:v>
       </x:c>
       <x:c r="H14" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I14" s="13" t="n">
-        <x:v>1262216.4</x:v>
+        <x:v>1252488.4</x:v>
       </x:c>
       <x:c r="J14" s="13" t="n">
         <x:v>0</x:v>
@@ -13144,16 +13144,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F15" s="13" t="n">
-        <x:v>12874080</x:v>
+        <x:v>12776800</x:v>
       </x:c>
       <x:c r="G15" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="H15" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I15" s="13" t="n">
-        <x:v>1287408</x:v>
+        <x:v>1277680</x:v>
       </x:c>
       <x:c r="J15" s="13" t="n">
         <x:v>0</x:v>
@@ -13183,10 +13183,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F16" s="13" t="n">
-        <x:v>8526835.3872</x:v>
+        <x:v>8419827.3872</x:v>
       </x:c>
       <x:c r="G16" s="13" t="n">
-        <x:v>8526835.3872</x:v>
+        <x:v>8419827.3872</x:v>
       </x:c>
       <x:c r="H16" s="13" t="n">
         <x:v>0</x:v>
@@ -13222,10 +13222,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F17" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="G17" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="H17" s="13" t="n">
         <x:v>0</x:v>
@@ -13261,16 +13261,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F18" s="13" t="n">
-        <x:v>7103892.6564</x:v>
+        <x:v>7006612.6564</x:v>
       </x:c>
       <x:c r="G18" s="13" t="n">
-        <x:v>8366109.0564</x:v>
+        <x:v>8259101.0564</x:v>
       </x:c>
       <x:c r="H18" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I18" s="13" t="n">
-        <x:v>1262216.4</x:v>
+        <x:v>1252488.4</x:v>
       </x:c>
       <x:c r="J18" s="13" t="n">
         <x:v>0</x:v>
@@ -13300,16 +13300,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F19" s="13" t="n">
-        <x:v>12874080</x:v>
+        <x:v>12776800</x:v>
       </x:c>
       <x:c r="G19" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="H19" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="13" t="n">
-        <x:v>1287408</x:v>
+        <x:v>1277680</x:v>
       </x:c>
       <x:c r="J19" s="13" t="n">
         <x:v>0</x:v>
@@ -13339,10 +13339,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F20" s="13" t="n">
-        <x:v>8366109.0564</x:v>
+        <x:v>8259101.0564</x:v>
       </x:c>
       <x:c r="G20" s="13" t="n">
-        <x:v>8366109.0564</x:v>
+        <x:v>8259101.0564</x:v>
       </x:c>
       <x:c r="H20" s="13" t="n">
         <x:v>0</x:v>
@@ -13378,10 +13378,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F21" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="G21" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="H21" s="13" t="n">
         <x:v>0</x:v>
@@ -13417,16 +13417,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F22" s="13" t="n">
-        <x:v>6938344.5216</x:v>
+        <x:v>6841064.5216</x:v>
       </x:c>
       <x:c r="G22" s="13" t="n">
-        <x:v>8200560.9216</x:v>
+        <x:v>8093552.9216</x:v>
       </x:c>
       <x:c r="H22" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I22" s="13" t="n">
-        <x:v>1262216.4</x:v>
+        <x:v>1252488.4</x:v>
       </x:c>
       <x:c r="J22" s="13" t="n">
         <x:v>0</x:v>
@@ -13456,16 +13456,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F23" s="13" t="n">
-        <x:v>12874080</x:v>
+        <x:v>12776800</x:v>
       </x:c>
       <x:c r="G23" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="H23" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I23" s="13" t="n">
-        <x:v>1287408</x:v>
+        <x:v>1277680</x:v>
       </x:c>
       <x:c r="J23" s="13" t="n">
         <x:v>0</x:v>
@@ -13495,10 +13495,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F24" s="13" t="n">
-        <x:v>8200560.9216</x:v>
+        <x:v>8093552.9216</x:v>
       </x:c>
       <x:c r="G24" s="13" t="n">
-        <x:v>8200560.9216</x:v>
+        <x:v>8093552.9216</x:v>
       </x:c>
       <x:c r="H24" s="13" t="n">
         <x:v>0</x:v>
@@ -13534,10 +13534,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F25" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="G25" s="13" t="n">
-        <x:v>14161488</x:v>
+        <x:v>14054480</x:v>
       </x:c>
       <x:c r="H25" s="13" t="n">
         <x:v>0</x:v>
@@ -22153,16 +22153,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F246" s="13" t="n">
-        <x:v>5487398.6048</x:v>
+        <x:v>5315773.6448</x:v>
       </x:c>
       <x:c r="G246" s="13" t="n">
-        <x:v>5880659.479</x:v>
+        <x:v>5706099.223</x:v>
       </x:c>
       <x:c r="H246" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I246" s="13" t="n">
-        <x:v>393260.8742</x:v>
+        <x:v>390325.5782</x:v>
       </x:c>
       <x:c r="J246" s="13" t="n">
         <x:v>0</x:v>
@@ -22172,7 +22172,7 @@
       </x:c>
       <x:c r="L246" s="14" t="n">
         <x:f>G246-F246-SUM(H246:K246)</x:f>
-        <x:v>4.0745362639427185e-10</x:v>
+        <x:v>3.4924596548080444e-10</x:v>
       </x:c>
     </x:row>
     <x:row r="247" ht="19" customHeight="1">
@@ -22192,16 +22192,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F247" s="13" t="n">
-        <x:v>10982400</x:v>
+        <x:v>10810176</x:v>
       </x:c>
       <x:c r="G247" s="13" t="n">
-        <x:v>11387500.8</x:v>
+        <x:v>11212281.6</x:v>
       </x:c>
       <x:c r="H247" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I247" s="13" t="n">
-        <x:v>405100.8</x:v>
+        <x:v>402105.6</x:v>
       </x:c>
       <x:c r="J247" s="13" t="n">
         <x:v>0</x:v>
@@ -22211,7 +22211,7 @@
       </x:c>
       <x:c r="L247" s="14" t="n">
         <x:f>G247-F247-SUM(H247:K247)</x:f>
-        <x:v>7.566995918750763e-10</x:v>
+        <x:v>-3.4924596548080444e-10</x:v>
       </x:c>
     </x:row>
     <x:row r="248" ht="19" customHeight="1">
@@ -22231,10 +22231,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F248" s="13" t="n">
-        <x:v>5880659.479</x:v>
+        <x:v>5706099.223</x:v>
       </x:c>
       <x:c r="G248" s="13" t="n">
-        <x:v>5880659.479</x:v>
+        <x:v>5706099.223</x:v>
       </x:c>
       <x:c r="H248" s="13" t="n">
         <x:v>0</x:v>
@@ -22270,10 +22270,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F249" s="13" t="n">
-        <x:v>11387500.8</x:v>
+        <x:v>11212281.6</x:v>
       </x:c>
       <x:c r="G249" s="13" t="n">
-        <x:v>11387500.8</x:v>
+        <x:v>11212281.6</x:v>
       </x:c>
       <x:c r="H249" s="13" t="n">
         <x:v>0</x:v>
@@ -22309,16 +22309,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F250" s="13" t="n">
-        <x:v>8596592.256</x:v>
+        <x:v>8312048.256</x:v>
       </x:c>
       <x:c r="G250" s="13" t="n">
-        <x:v>9997207.4803</x:v>
+        <x:v>9684209.0803</x:v>
       </x:c>
       <x:c r="H250" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I250" s="13" t="n">
-        <x:v>1400615.2243</x:v>
+        <x:v>1372160.8243</x:v>
       </x:c>
       <x:c r="J250" s="13" t="n">
         <x:v>0</x:v>
@@ -22328,7 +22328,7 @@
       </x:c>
       <x:c r="L250" s="14" t="n">
         <x:f>G250-F250-SUM(H250:K250)</x:f>
-        <x:v>9.313225746154785e-10</x:v>
+        <x:v>-4.656612873077393e-10</x:v>
       </x:c>
     </x:row>
     <x:row r="251" ht="19" customHeight="1">
@@ -22348,16 +22348,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F251" s="13" t="n">
-        <x:v>14299584</x:v>
+        <x:v>14015040</x:v>
       </x:c>
       <x:c r="G251" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="H251" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I251" s="13" t="n">
-        <x:v>1429958.4</x:v>
+        <x:v>1401504</x:v>
       </x:c>
       <x:c r="J251" s="13" t="n">
         <x:v>0</x:v>
@@ -22367,7 +22367,7 @@
       </x:c>
       <x:c r="L251" s="14" t="n">
         <x:f>G251-F251-SUM(H251:K251)</x:f>
-        <x:v>4.656612873077393e-10</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="252" ht="19" customHeight="1">
@@ -22387,10 +22387,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F252" s="13" t="n">
-        <x:v>9997207.4803</x:v>
+        <x:v>9684209.0803</x:v>
       </x:c>
       <x:c r="G252" s="13" t="n">
-        <x:v>9997207.4803</x:v>
+        <x:v>9684209.0803</x:v>
       </x:c>
       <x:c r="H252" s="13" t="n">
         <x:v>0</x:v>
@@ -22426,10 +22426,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F253" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="G253" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="H253" s="13" t="n">
         <x:v>0</x:v>
@@ -22465,16 +22465,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F254" s="13" t="n">
-        <x:v>8434305.456</x:v>
+        <x:v>8149761.456</x:v>
       </x:c>
       <x:c r="G254" s="13" t="n">
-        <x:v>9834920.6803</x:v>
+        <x:v>9521922.2803</x:v>
       </x:c>
       <x:c r="H254" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I254" s="13" t="n">
-        <x:v>1400615.2243</x:v>
+        <x:v>1372160.8243</x:v>
       </x:c>
       <x:c r="J254" s="13" t="n">
         <x:v>0</x:v>
@@ -22484,7 +22484,7 @@
       </x:c>
       <x:c r="L254" s="14" t="n">
         <x:f>G254-F254-SUM(H254:K254)</x:f>
-        <x:v>-9.313225746154785e-10</x:v>
+        <x:v>4.656612873077393e-10</x:v>
       </x:c>
     </x:row>
     <x:row r="255" ht="19" customHeight="1">
@@ -22504,16 +22504,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F255" s="13" t="n">
-        <x:v>14299584</x:v>
+        <x:v>14015040</x:v>
       </x:c>
       <x:c r="G255" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="H255" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I255" s="13" t="n">
-        <x:v>1429958.4</x:v>
+        <x:v>1401504</x:v>
       </x:c>
       <x:c r="J255" s="13" t="n">
         <x:v>0</x:v>
@@ -22523,7 +22523,7 @@
       </x:c>
       <x:c r="L255" s="14" t="n">
         <x:f>G255-F255-SUM(H255:K255)</x:f>
-        <x:v>4.656612873077393e-10</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="256" ht="19" customHeight="1">
@@ -22543,10 +22543,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F256" s="13" t="n">
-        <x:v>9834920.6803</x:v>
+        <x:v>9521922.2803</x:v>
       </x:c>
       <x:c r="G256" s="13" t="n">
-        <x:v>9834920.6803</x:v>
+        <x:v>9521922.2803</x:v>
       </x:c>
       <x:c r="H256" s="13" t="n">
         <x:v>0</x:v>
@@ -22582,10 +22582,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F257" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="G257" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="H257" s="13" t="n">
         <x:v>0</x:v>
@@ -22621,16 +22621,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F258" s="13" t="n">
-        <x:v>8267150.052</x:v>
+        <x:v>7982606.052</x:v>
       </x:c>
       <x:c r="G258" s="13" t="n">
-        <x:v>9667765.2763</x:v>
+        <x:v>9354766.8763</x:v>
       </x:c>
       <x:c r="H258" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I258" s="13" t="n">
-        <x:v>1400615.2243</x:v>
+        <x:v>1372160.8243</x:v>
       </x:c>
       <x:c r="J258" s="13" t="n">
         <x:v>0</x:v>
@@ -22640,7 +22640,7 @@
       </x:c>
       <x:c r="L258" s="14" t="n">
         <x:f>G258-F258-SUM(H258:K258)</x:f>
-        <x:v>0</x:v>
+        <x:v>-4.656612873077393e-10</x:v>
       </x:c>
     </x:row>
     <x:row r="259" ht="19" customHeight="1">
@@ -22660,16 +22660,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F259" s="13" t="n">
-        <x:v>14299584</x:v>
+        <x:v>14015040</x:v>
       </x:c>
       <x:c r="G259" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="H259" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I259" s="13" t="n">
-        <x:v>1429958.4</x:v>
+        <x:v>1401504</x:v>
       </x:c>
       <x:c r="J259" s="13" t="n">
         <x:v>0</x:v>
@@ -22679,7 +22679,7 @@
       </x:c>
       <x:c r="L259" s="14" t="n">
         <x:f>G259-F259-SUM(H259:K259)</x:f>
-        <x:v>4.656612873077393e-10</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="260" ht="19" customHeight="1">
@@ -22699,10 +22699,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F260" s="13" t="n">
-        <x:v>9667765.2763</x:v>
+        <x:v>9354766.8763</x:v>
       </x:c>
       <x:c r="G260" s="13" t="n">
-        <x:v>9667765.2763</x:v>
+        <x:v>9354766.8763</x:v>
       </x:c>
       <x:c r="H260" s="13" t="n">
         <x:v>0</x:v>
@@ -22738,10 +22738,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F261" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="G261" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="H261" s="13" t="n">
         <x:v>0</x:v>
@@ -22777,16 +22777,16 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F262" s="13" t="n">
-        <x:v>8094979.9788</x:v>
+        <x:v>7810435.9788</x:v>
       </x:c>
       <x:c r="G262" s="13" t="n">
-        <x:v>9495595.2031</x:v>
+        <x:v>9182596.8031</x:v>
       </x:c>
       <x:c r="H262" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I262" s="13" t="n">
-        <x:v>1400615.2243</x:v>
+        <x:v>1372160.8243</x:v>
       </x:c>
       <x:c r="J262" s="13" t="n">
         <x:v>0</x:v>
@@ -22796,7 +22796,7 @@
       </x:c>
       <x:c r="L262" s="14" t="n">
         <x:f>G262-F262-SUM(H262:K262)</x:f>
-        <x:v>0</x:v>
+        <x:v>-4.656612873077393e-10</x:v>
       </x:c>
     </x:row>
     <x:row r="263" ht="19" customHeight="1">
@@ -22816,16 +22816,16 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F263" s="13" t="n">
-        <x:v>14299584</x:v>
+        <x:v>14015040</x:v>
       </x:c>
       <x:c r="G263" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="H263" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I263" s="13" t="n">
-        <x:v>1429958.4</x:v>
+        <x:v>1401504</x:v>
       </x:c>
       <x:c r="J263" s="13" t="n">
         <x:v>0</x:v>
@@ -22835,7 +22835,7 @@
       </x:c>
       <x:c r="L263" s="14" t="n">
         <x:f>G263-F263-SUM(H263:K263)</x:f>
-        <x:v>4.656612873077393e-10</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="264" ht="19" customHeight="1">
@@ -22855,10 +22855,10 @@
         <x:v>net_income_usd</x:v>
       </x:c>
       <x:c r="F264" s="13" t="n">
-        <x:v>9495595.2031</x:v>
+        <x:v>9182596.8031</x:v>
       </x:c>
       <x:c r="G264" s="13" t="n">
-        <x:v>9495595.2031</x:v>
+        <x:v>9182596.8031</x:v>
       </x:c>
       <x:c r="H264" s="13" t="n">
         <x:v>0</x:v>
@@ -22894,10 +22894,10 @@
         <x:v>revenue_usd</x:v>
       </x:c>
       <x:c r="F265" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="G265" s="13" t="n">
-        <x:v>15729542.4</x:v>
+        <x:v>15416544</x:v>
       </x:c>
       <x:c r="H265" s="13" t="n">
         <x:v>0</x:v>

</xml_diff>